<commit_message>
11/03/2026 - Observaciones atendidas 2.0
</commit_message>
<xml_diff>
--- a/plantillas/consulta/Base_Datos.xlsx
+++ b/plantillas/consulta/Base_Datos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Visual Studio Code\NodeJS\SIVACC\plantillas\consulta\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{912995B2-CB14-4FF3-B43F-36AA058AC722}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D58AB8CD-7726-4B19-BA45-9D306FDD550E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -71,9 +71,6 @@
     <t>Nombre de la Unidad Territorial</t>
   </si>
   <si>
-    <t>Rubro General o Destino</t>
-  </si>
-  <si>
     <t>Mesa</t>
   </si>
   <si>
@@ -94,6 +91,9 @@
   <si>
     <t>SISTEMA DE CÓMPUTO Y VALIDACIONES PARA LAS CONSULTAS CIUDADANAS
 SICOVACC 2026</t>
+  </si>
+  <si>
+    <t>Destino de los recursos</t>
   </si>
 </sst>
 </file>
@@ -230,9 +230,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -246,6 +243,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -595,86 +595,86 @@
       <c r="M1" s="4"/>
     </row>
     <row r="2" spans="1:13" ht="20.25" x14ac:dyDescent="0.2">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
-      <c r="H2" s="13"/>
-      <c r="I2" s="13"/>
-      <c r="J2" s="13"/>
-      <c r="K2" s="13"/>
-      <c r="L2" s="13"/>
-      <c r="M2" s="13"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
+      <c r="M2" s="12"/>
     </row>
     <row r="3" spans="1:13" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3" s="15"/>
-      <c r="C3" s="15"/>
-      <c r="D3" s="15"/>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15"/>
-      <c r="G3" s="15"/>
-      <c r="H3" s="15"/>
-      <c r="I3" s="15"/>
-      <c r="J3" s="15"/>
-      <c r="K3" s="15"/>
-      <c r="L3" s="15"/>
-      <c r="M3" s="15"/>
+      <c r="A3" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
+      <c r="I3" s="14"/>
+      <c r="J3" s="14"/>
+      <c r="K3" s="14"/>
+      <c r="L3" s="14"/>
+      <c r="M3" s="14"/>
     </row>
     <row r="4" spans="1:13" ht="15" x14ac:dyDescent="0.2">
-      <c r="A4" s="16"/>
-      <c r="B4" s="16"/>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="16"/>
-      <c r="G4" s="16"/>
-      <c r="H4" s="16"/>
-      <c r="I4" s="16"/>
-      <c r="J4" s="16"/>
-      <c r="K4" s="16"/>
-      <c r="L4" s="16"/>
+      <c r="A4" s="15"/>
+      <c r="B4" s="15"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="15"/>
+      <c r="H4" s="15"/>
+      <c r="I4" s="15"/>
+      <c r="J4" s="15"/>
+      <c r="K4" s="15"/>
+      <c r="L4" s="15"/>
     </row>
     <row r="5" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" s="14"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14"/>
-      <c r="G5" s="14"/>
-      <c r="H5" s="14"/>
-      <c r="I5" s="14"/>
-      <c r="J5" s="14"/>
-      <c r="K5" s="14"/>
-      <c r="L5" s="14"/>
-      <c r="M5" s="14"/>
+      <c r="A5" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="13"/>
+      <c r="G5" s="13"/>
+      <c r="H5" s="13"/>
+      <c r="I5" s="13"/>
+      <c r="J5" s="13"/>
+      <c r="K5" s="13"/>
+      <c r="L5" s="13"/>
+      <c r="M5" s="13"/>
     </row>
     <row r="6" spans="1:13" ht="18" x14ac:dyDescent="0.2">
-      <c r="A6" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" s="15"/>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="15"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
-      <c r="I6" s="15"/>
-      <c r="J6" s="15"/>
-      <c r="K6" s="15"/>
-      <c r="L6" s="15"/>
-      <c r="M6" s="15"/>
+      <c r="A6" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="14"/>
+      <c r="C6" s="14"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
+      <c r="I6" s="14"/>
+      <c r="J6" s="14"/>
+      <c r="K6" s="14"/>
+      <c r="L6" s="14"/>
+      <c r="M6" s="14"/>
     </row>
     <row r="7" spans="1:13" ht="15" x14ac:dyDescent="0.2">
       <c r="A7" s="9"/>
@@ -702,64 +702,64 @@
       <c r="M9" s="11"/>
     </row>
     <row r="11" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="12" t="s">
+      <c r="A11" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="B11" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="C11" s="12" t="s">
-        <v>16</v>
-      </c>
-      <c r="D11" s="12" t="s">
+      <c r="C11" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="E11" s="12" t="s">
+      <c r="E11" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="F11" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="G11" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="H11" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="I11" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="K11" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="F11" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="G11" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H11" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="I11" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="J11" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="K11" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="L11" s="12" t="s">
+      <c r="L11" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="M11" s="12" t="s">
+      <c r="M11" s="17" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="12"/>
-      <c r="B12" s="12"/>
-      <c r="C12" s="12"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="12"/>
-      <c r="F12" s="12"/>
-      <c r="G12" s="12"/>
-      <c r="H12" s="12"/>
-      <c r="I12" s="12"/>
+      <c r="A12" s="17"/>
+      <c r="B12" s="17"/>
+      <c r="C12" s="17"/>
+      <c r="D12" s="17"/>
+      <c r="E12" s="17"/>
+      <c r="F12" s="17"/>
+      <c r="G12" s="17"/>
+      <c r="H12" s="17"/>
+      <c r="I12" s="17"/>
       <c r="J12" s="7" t="s">
         <v>2</v>
       </c>
       <c r="K12" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="L12" s="12"/>
-      <c r="M12" s="12"/>
+      <c r="L12" s="17"/>
+      <c r="M12" s="17"/>
     </row>
     <row r="13" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="5"/>
@@ -778,22 +778,22 @@
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A5:M5"/>
-    <mergeCell ref="A6:M6"/>
-    <mergeCell ref="A4:L4"/>
-    <mergeCell ref="A3:M3"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
     <mergeCell ref="M11:M12"/>
     <mergeCell ref="F11:F12"/>
     <mergeCell ref="G11:G12"/>
     <mergeCell ref="H11:H12"/>
     <mergeCell ref="I11:I12"/>
     <mergeCell ref="L11:L12"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A5:M5"/>
+    <mergeCell ref="A6:M6"/>
+    <mergeCell ref="A4:L4"/>
+    <mergeCell ref="A3:M3"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="40" fitToHeight="0" orientation="landscape" r:id="rId1"/>

</xml_diff>